<commit_message>
refactor: rename function column to keyword
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Final Excel Template.xlsx
+++ b/src/test/resources/testdata/Final Excel Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\seleniumAutomationSystem\src\test\resources\testdata\"/>
     </mc:Choice>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="115">
   <si>
     <t>NO</t>
   </si>
@@ -369,12 +369,16 @@
   </si>
   <si>
     <t>HRIS login button</t>
+  </si>
+  <si>
+    <t>Keyword</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -607,11 +611,11 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="36.875" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="3.625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="4.75"/>
+    <col min="3" max="3" customWidth="true" style="2" width="25.625"/>
+    <col min="4" max="4" customWidth="true" style="2" width="36.875"/>
+    <col min="5" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -683,9 +687,9 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="48.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="3.75"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="48.375"/>
+    <col min="3" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -733,10 +737,10 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="3.375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="13.375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="2" width="9.875"/>
+    <col min="4" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -796,12 +800,12 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="3.375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="16.375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="2" width="13.875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="2" width="24.875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="2" width="10.875"/>
+    <col min="6" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -882,13 +886,13 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.25" customWidth="1"/>
-    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="16.125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="4.5"/>
+    <col min="3" max="3" customWidth="true" width="27.25"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="17.5"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="36.25"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="10.625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="19.75"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
@@ -899,7 +903,7 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>18</v>
@@ -1133,14 +1137,14 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="13.5"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="4.5"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="2" width="13.25"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="2" width="17.5"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="2" width="36.25"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="2" width="10.625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="2" width="15.375"/>
+    <col min="8" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1151,7 +1155,7 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>18</v>
@@ -1313,14 +1317,14 @@
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="13.75"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="4.5"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="2" width="8.625"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="2" width="17.5"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="2" width="36.25"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="2" width="10.625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" style="2" width="14.625"/>
+    <col min="8" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1331,7 +1335,7 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>18</v>
@@ -1471,11 +1475,11 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="2"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" style="2" width="15.625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="2" width="34.875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" style="2" width="9.75"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" style="2" width="25.5"/>
+    <col min="5" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">

</xml_diff>